<commit_message>
Rebuild the Bayes worksheet on the widened hitter prior
The base rate the worksheet's given cells quote now comes from hitters in a band around
the subject's own career average rather than everyone at or below a ceiling, so the prior
a student is handed is the base rate for a hitter like the one in the problem.
</commit_message>
<xml_diff>
--- a/weeks/week03/data/hand-build-bayes-worksheet.xlsx
+++ b/weeks/week03/data/hand-build-bayes-worksheet.xlsx
@@ -474,7 +474,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>LaMonte Wade Jr.</t>
+          <t>Salvador Perez</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -496,7 +496,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1077</v>
+        <v>5290</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
@@ -548,7 +548,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>260</v>
+        <v>1411</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
@@ -565,7 +565,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>63</v>
+        <v>107</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>0.0212</v>
+        <v>0.0509</v>
       </c>
     </row>
     <row r="11">

</xml_diff>